<commit_message>
added models Ref Lokasi
</commit_message>
<xml_diff>
--- a/ref/Referensi-Jabatan-Struktural (2) (1).xlsx
+++ b/ref/Referensi-Jabatan-Struktural (2) (1).xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="11008"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B269C120-3662-0B42-94BB-0EEE3ACD1932}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4767AD87-2D30-D347-A512-0227EA2DBA29}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="15800" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -13819,8 +13819,8 @@
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="36.6640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="105.1640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="111.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="77.1640625" customWidth="1"/>
+    <col min="3" max="3" width="55.83203125" customWidth="1"/>
     <col min="4" max="4" width="8.83203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>

</xml_diff>